<commit_message>
update export DNTU and create product from SO
</commit_message>
<xml_diff>
--- a/SourceCode/EV_ERP/EV_ERP/wwwroot/templates/DNHU-template.xlsx
+++ b/SourceCode/EV_ERP/EV_ERP/wwwroot/templates/DNHU-template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Dev\EV_ERP_History\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Dev\EV_ERP\SourceCode\EV_ERP\EV_ERP\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC9F6DBA-DC9F-4EF3-83A0-34D42801FADB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9976209-8205-4CD0-BFE5-F62B5FFBFF83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1461,6 +1461,57 @@
     <xf numFmtId="166" fontId="15" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="43" fontId="19" fillId="13" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="28" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="14" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="14" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="9" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="9" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="9" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="9" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="9" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="9" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="27" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="27" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="18" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1470,8 +1521,50 @@
     <xf numFmtId="166" fontId="23" fillId="7" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="15" fillId="4" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="4" borderId="11" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="16" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="11" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="15" fillId="11" borderId="2" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="3" fontId="15" fillId="5" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="33" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="34" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="3" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="21" fillId="6" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="166" fontId="25" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -1503,12 +1596,6 @@
     <xf numFmtId="166" fontId="22" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="14" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="14" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="25" fillId="12" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1530,98 +1617,11 @@
     <xf numFmtId="166" fontId="22" fillId="8" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="27" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="27" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="15" fillId="0" borderId="3" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="15" fillId="0" borderId="5" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="33" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="34" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="20" fillId="3" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="21" fillId="6" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="11" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="15" fillId="11" borderId="2" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="22" fillId="9" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="22" fillId="9" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="22" fillId="9" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="22" fillId="9" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="22" fillId="9" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="22" fillId="9" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="4" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="4" borderId="11" xfId="4" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="16" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="19" fillId="13" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="28" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -2035,25 +2035,25 @@
       <c r="C1" s="1"/>
       <c r="E1" s="71"/>
       <c r="F1" s="14"/>
-      <c r="G1" s="173" t="s">
+      <c r="G1" s="175" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="173"/>
-      <c r="I1" s="173"/>
-      <c r="J1" s="173"/>
-      <c r="K1" s="173"/>
-      <c r="L1" s="173"/>
-      <c r="M1" s="173"/>
-      <c r="N1" s="173"/>
-      <c r="O1" s="173"/>
-      <c r="P1" s="173"/>
-      <c r="Q1" s="173"/>
-      <c r="R1" s="173"/>
-      <c r="S1" s="173"/>
-      <c r="T1" s="173"/>
-      <c r="U1" s="173"/>
-      <c r="V1" s="173"/>
-      <c r="W1" s="173"/>
+      <c r="H1" s="175"/>
+      <c r="I1" s="175"/>
+      <c r="J1" s="175"/>
+      <c r="K1" s="175"/>
+      <c r="L1" s="175"/>
+      <c r="M1" s="175"/>
+      <c r="N1" s="175"/>
+      <c r="O1" s="175"/>
+      <c r="P1" s="175"/>
+      <c r="Q1" s="175"/>
+      <c r="R1" s="175"/>
+      <c r="S1" s="175"/>
+      <c r="T1" s="175"/>
+      <c r="U1" s="175"/>
+      <c r="V1" s="175"/>
+      <c r="W1" s="175"/>
     </row>
     <row r="2" spans="1:23" ht="55.95" customHeight="1">
       <c r="A2" s="1"/>
@@ -2061,25 +2061,25 @@
       <c r="C2" s="1"/>
       <c r="E2" s="13"/>
       <c r="F2" s="12"/>
-      <c r="G2" s="174" t="s">
+      <c r="G2" s="176" t="s">
         <v>49</v>
       </c>
-      <c r="H2" s="174"/>
-      <c r="I2" s="174"/>
-      <c r="J2" s="174"/>
-      <c r="K2" s="174"/>
-      <c r="L2" s="174"/>
-      <c r="M2" s="174"/>
-      <c r="N2" s="174"/>
-      <c r="O2" s="174"/>
-      <c r="P2" s="174"/>
-      <c r="Q2" s="174"/>
-      <c r="R2" s="174"/>
-      <c r="S2" s="174"/>
-      <c r="T2" s="174"/>
-      <c r="U2" s="174"/>
-      <c r="V2" s="174"/>
-      <c r="W2" s="174"/>
+      <c r="H2" s="176"/>
+      <c r="I2" s="176"/>
+      <c r="J2" s="176"/>
+      <c r="K2" s="176"/>
+      <c r="L2" s="176"/>
+      <c r="M2" s="176"/>
+      <c r="N2" s="176"/>
+      <c r="O2" s="176"/>
+      <c r="P2" s="176"/>
+      <c r="Q2" s="176"/>
+      <c r="R2" s="176"/>
+      <c r="S2" s="176"/>
+      <c r="T2" s="176"/>
+      <c r="U2" s="176"/>
+      <c r="V2" s="176"/>
+      <c r="W2" s="176"/>
     </row>
     <row r="3" spans="1:23" ht="64.5" customHeight="1">
       <c r="A3" s="1"/>
@@ -2087,52 +2087,52 @@
       <c r="C3" s="1"/>
       <c r="E3" s="13"/>
       <c r="F3" s="12"/>
-      <c r="G3" s="174" t="s">
+      <c r="G3" s="176" t="s">
         <v>1</v>
       </c>
-      <c r="H3" s="174"/>
-      <c r="I3" s="174"/>
-      <c r="J3" s="174"/>
-      <c r="K3" s="174"/>
-      <c r="L3" s="174"/>
-      <c r="M3" s="174"/>
-      <c r="N3" s="174"/>
-      <c r="O3" s="174"/>
-      <c r="P3" s="174"/>
-      <c r="Q3" s="174"/>
-      <c r="R3" s="174"/>
-      <c r="S3" s="174"/>
-      <c r="T3" s="174"/>
-      <c r="U3" s="174"/>
-      <c r="V3" s="174"/>
-      <c r="W3" s="174"/>
+      <c r="H3" s="176"/>
+      <c r="I3" s="176"/>
+      <c r="J3" s="176"/>
+      <c r="K3" s="176"/>
+      <c r="L3" s="176"/>
+      <c r="M3" s="176"/>
+      <c r="N3" s="176"/>
+      <c r="O3" s="176"/>
+      <c r="P3" s="176"/>
+      <c r="Q3" s="176"/>
+      <c r="R3" s="176"/>
+      <c r="S3" s="176"/>
+      <c r="T3" s="176"/>
+      <c r="U3" s="176"/>
+      <c r="V3" s="176"/>
+      <c r="W3" s="176"/>
     </row>
     <row r="4" spans="1:23" ht="75.75" customHeight="1">
-      <c r="A4" s="175" t="s">
+      <c r="A4" s="177" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="175"/>
-      <c r="C4" s="175"/>
-      <c r="D4" s="175"/>
-      <c r="E4" s="175"/>
-      <c r="F4" s="175"/>
-      <c r="G4" s="175"/>
-      <c r="H4" s="175"/>
-      <c r="I4" s="175"/>
-      <c r="J4" s="175"/>
-      <c r="K4" s="175"/>
-      <c r="L4" s="175"/>
-      <c r="M4" s="175"/>
-      <c r="N4" s="175"/>
-      <c r="O4" s="175"/>
-      <c r="P4" s="175"/>
-      <c r="Q4" s="175"/>
-      <c r="R4" s="175"/>
-      <c r="S4" s="175"/>
-      <c r="T4" s="175"/>
-      <c r="U4" s="175"/>
-      <c r="V4" s="175"/>
-      <c r="W4" s="175"/>
+      <c r="B4" s="177"/>
+      <c r="C4" s="177"/>
+      <c r="D4" s="177"/>
+      <c r="E4" s="177"/>
+      <c r="F4" s="177"/>
+      <c r="G4" s="177"/>
+      <c r="H4" s="177"/>
+      <c r="I4" s="177"/>
+      <c r="J4" s="177"/>
+      <c r="K4" s="177"/>
+      <c r="L4" s="177"/>
+      <c r="M4" s="177"/>
+      <c r="N4" s="177"/>
+      <c r="O4" s="177"/>
+      <c r="P4" s="177"/>
+      <c r="Q4" s="177"/>
+      <c r="R4" s="177"/>
+      <c r="S4" s="177"/>
+      <c r="T4" s="177"/>
+      <c r="U4" s="177"/>
+      <c r="V4" s="177"/>
+      <c r="W4" s="177"/>
     </row>
     <row r="5" spans="1:23" s="4" customFormat="1">
       <c r="A5" s="15" t="s">
@@ -2142,22 +2142,19 @@
       <c r="C5" s="15"/>
       <c r="D5" s="15"/>
       <c r="E5" s="86"/>
-      <c r="F5" s="178" t="s">
+      <c r="F5" s="180" t="s">
         <v>44</v>
       </c>
-      <c r="G5" s="178"/>
-      <c r="H5" s="178"/>
-      <c r="I5" s="177" t="e">
-        <f>+#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="J5" s="177"/>
-      <c r="K5" s="176" t="s">
+      <c r="G5" s="180"/>
+      <c r="H5" s="180"/>
+      <c r="I5" s="179"/>
+      <c r="J5" s="179"/>
+      <c r="K5" s="178" t="s">
         <v>39</v>
       </c>
-      <c r="L5" s="176"/>
-      <c r="M5" s="176"/>
-      <c r="N5" s="176"/>
+      <c r="L5" s="178"/>
+      <c r="M5" s="178"/>
+      <c r="N5" s="178"/>
       <c r="O5" s="46"/>
       <c r="P5" s="86"/>
       <c r="Q5" s="18"/>
@@ -2299,13 +2296,13 @@
         <f>+#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="D10" s="179" t="s">
+      <c r="D10" s="171" t="s">
         <v>45</v>
       </c>
-      <c r="E10" s="179"/>
-      <c r="F10" s="179"/>
-      <c r="G10" s="180"/>
-      <c r="H10" s="180"/>
+      <c r="E10" s="171"/>
+      <c r="F10" s="171"/>
+      <c r="G10" s="172"/>
+      <c r="H10" s="172"/>
       <c r="I10" s="94"/>
       <c r="J10" s="94"/>
       <c r="K10" s="94"/>
@@ -2478,16 +2475,16 @@
     </row>
     <row r="13" spans="1:23" s="1" customFormat="1" ht="71.25" customHeight="1">
       <c r="A13" s="48"/>
-      <c r="B13" s="181" t="s">
+      <c r="B13" s="173" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="181"/>
-      <c r="D13" s="181"/>
-      <c r="E13" s="149" t="e">
+      <c r="C13" s="173"/>
+      <c r="D13" s="173"/>
+      <c r="E13" s="174" t="e">
         <f>SUMPRODUCT($E$12:E12,F12:F12)</f>
         <v>#REF!</v>
       </c>
-      <c r="F13" s="149"/>
+      <c r="F13" s="174"/>
       <c r="G13" s="72" t="e">
         <f>SUMPRODUCT(E12:E12,F12:F12,G12:G12)</f>
         <v>#REF!</v>
@@ -2497,15 +2494,15 @@
         <v>#REF!</v>
       </c>
       <c r="I13" s="50"/>
-      <c r="J13" s="181" t="s">
+      <c r="J13" s="173" t="s">
         <v>24</v>
       </c>
-      <c r="K13" s="181"/>
-      <c r="L13" s="149" t="e">
+      <c r="K13" s="173"/>
+      <c r="L13" s="174" t="e">
         <f>SUMPRODUCT(L12:L12,M12:M12)</f>
         <v>#REF!</v>
       </c>
-      <c r="M13" s="149"/>
+      <c r="M13" s="174"/>
       <c r="N13" s="72" t="e">
         <f>SUMPRODUCT(L12:L12,M12:M12,N12:N12)</f>
         <v>#REF!</v>
@@ -2538,13 +2535,13 @@
     <row r="14" spans="1:23" ht="46.95" customHeight="1">
       <c r="A14" s="51"/>
       <c r="B14" s="51"/>
-      <c r="C14" s="150"/>
-      <c r="D14" s="151"/>
-      <c r="E14" s="162">
+      <c r="C14" s="181"/>
+      <c r="D14" s="182"/>
+      <c r="E14" s="191">
         <f>SUMIF(N12:N12,"0",H12:H12)</f>
         <v>0</v>
       </c>
-      <c r="F14" s="162"/>
+      <c r="F14" s="191"/>
       <c r="G14" s="109" t="s">
         <v>26</v>
       </c>
@@ -2553,15 +2550,15 @@
         <v>#REF!</v>
       </c>
       <c r="I14" s="111"/>
-      <c r="J14" s="163" t="s">
+      <c r="J14" s="192" t="s">
         <v>31</v>
       </c>
-      <c r="K14" s="164"/>
-      <c r="L14" s="165"/>
-      <c r="M14" s="169" t="s">
+      <c r="K14" s="193"/>
+      <c r="L14" s="194"/>
+      <c r="M14" s="161" t="s">
         <v>28</v>
       </c>
-      <c r="N14" s="170"/>
+      <c r="N14" s="162"/>
       <c r="O14" s="128" t="e">
         <f>O13</f>
         <v>#REF!</v>
@@ -2569,10 +2566,10 @@
       <c r="P14" s="127" t="s">
         <v>22</v>
       </c>
-      <c r="Q14" s="146" t="s">
+      <c r="Q14" s="163" t="s">
         <v>42</v>
       </c>
-      <c r="R14" s="147"/>
+      <c r="R14" s="164"/>
       <c r="S14" s="128"/>
       <c r="T14" s="134" t="s">
         <v>22</v>
@@ -2590,21 +2587,21 @@
       <c r="G15" s="54"/>
       <c r="H15" s="55"/>
       <c r="I15" s="111"/>
-      <c r="J15" s="166"/>
-      <c r="K15" s="167"/>
-      <c r="L15" s="168"/>
-      <c r="M15" s="148" t="s">
+      <c r="J15" s="195"/>
+      <c r="K15" s="196"/>
+      <c r="L15" s="197"/>
+      <c r="M15" s="165" t="s">
         <v>40</v>
       </c>
-      <c r="N15" s="148"/>
+      <c r="N15" s="165"/>
       <c r="O15" s="107"/>
       <c r="P15" s="108" t="s">
         <v>22</v>
       </c>
-      <c r="Q15" s="160" t="s">
+      <c r="Q15" s="153" t="s">
         <v>46</v>
       </c>
-      <c r="R15" s="161"/>
+      <c r="R15" s="154"/>
       <c r="S15" s="107"/>
       <c r="T15" s="108" t="s">
         <v>22</v>
@@ -2622,23 +2619,23 @@
       <c r="G16" s="54"/>
       <c r="H16" s="55"/>
       <c r="I16" s="111"/>
-      <c r="J16" s="185" t="s">
+      <c r="J16" s="155" t="s">
         <v>32</v>
       </c>
-      <c r="K16" s="186"/>
-      <c r="L16" s="187"/>
-      <c r="M16" s="169" t="s">
+      <c r="K16" s="156"/>
+      <c r="L16" s="157"/>
+      <c r="M16" s="161" t="s">
         <v>28</v>
       </c>
-      <c r="N16" s="170"/>
+      <c r="N16" s="162"/>
       <c r="O16" s="128"/>
       <c r="P16" s="127" t="s">
         <v>22</v>
       </c>
-      <c r="Q16" s="146" t="s">
+      <c r="Q16" s="163" t="s">
         <v>42</v>
       </c>
-      <c r="R16" s="147"/>
+      <c r="R16" s="164"/>
       <c r="S16" s="128"/>
       <c r="T16" s="127" t="s">
         <v>22</v>
@@ -2656,21 +2653,21 @@
       <c r="G17" s="54"/>
       <c r="H17" s="55"/>
       <c r="I17" s="111"/>
-      <c r="J17" s="188"/>
-      <c r="K17" s="189"/>
-      <c r="L17" s="190"/>
-      <c r="M17" s="148" t="s">
+      <c r="J17" s="158"/>
+      <c r="K17" s="159"/>
+      <c r="L17" s="160"/>
+      <c r="M17" s="165" t="s">
         <v>40</v>
       </c>
-      <c r="N17" s="148"/>
+      <c r="N17" s="165"/>
       <c r="O17" s="107"/>
       <c r="P17" s="108" t="s">
         <v>22</v>
       </c>
-      <c r="Q17" s="160" t="s">
+      <c r="Q17" s="153" t="s">
         <v>46</v>
       </c>
-      <c r="R17" s="161"/>
+      <c r="R17" s="154"/>
       <c r="S17" s="107"/>
       <c r="T17" s="108" t="s">
         <v>22</v>
@@ -2691,18 +2688,18 @@
       <c r="J18" s="139"/>
       <c r="K18" s="139"/>
       <c r="L18" s="139"/>
-      <c r="M18" s="171" t="s">
+      <c r="M18" s="198" t="s">
         <v>59</v>
       </c>
-      <c r="N18" s="172"/>
+      <c r="N18" s="199"/>
       <c r="O18" s="144"/>
       <c r="P18" s="145" t="s">
         <v>22</v>
       </c>
-      <c r="Q18" s="195" t="s">
+      <c r="Q18" s="170" t="s">
         <v>55</v>
       </c>
-      <c r="R18" s="195"/>
+      <c r="R18" s="170"/>
       <c r="S18" s="128">
         <f>R13-50000</f>
         <v>200000</v>
@@ -2713,8 +2710,8 @@
       <c r="U18" s="138" t="s">
         <v>56</v>
       </c>
-      <c r="V18" s="196"/>
-      <c r="W18" s="196"/>
+      <c r="V18" s="146"/>
+      <c r="W18" s="146"/>
     </row>
     <row r="19" spans="1:23" ht="21.6" customHeight="1">
       <c r="A19" s="51"/>
@@ -2743,11 +2740,11 @@
     </row>
     <row r="20" spans="1:23" ht="44.4" customHeight="1">
       <c r="B20" s="59"/>
-      <c r="C20" s="156" t="s">
+      <c r="C20" s="187" t="s">
         <v>37</v>
       </c>
-      <c r="D20" s="156"/>
-      <c r="E20" s="157"/>
+      <c r="D20" s="187"/>
+      <c r="E20" s="188"/>
       <c r="F20" s="112" t="e">
         <f>+O14+O15</f>
         <v>#REF!</v>
@@ -2776,11 +2773,11 @@
     </row>
     <row r="21" spans="1:23" ht="44.4" customHeight="1">
       <c r="B21" s="59"/>
-      <c r="C21" s="158" t="s">
+      <c r="C21" s="189" t="s">
         <v>38</v>
       </c>
-      <c r="D21" s="158"/>
-      <c r="E21" s="159"/>
+      <c r="D21" s="189"/>
+      <c r="E21" s="190"/>
       <c r="F21" s="112">
         <f>+O16+O17</f>
         <v>0</v>
@@ -2809,14 +2806,14 @@
     </row>
     <row r="22" spans="1:23" ht="45.75" customHeight="1">
       <c r="B22" s="59"/>
-      <c r="C22" s="193" t="s">
+      <c r="C22" s="168" t="s">
         <v>47</v>
       </c>
-      <c r="D22" s="194" t="e">
+      <c r="D22" s="169" t="e">
         <f>T13-F20-F21</f>
         <v>#REF!</v>
       </c>
-      <c r="E22" s="194"/>
+      <c r="E22" s="169"/>
       <c r="F22" s="58" t="e">
         <f>T13-F20-F21-R13</f>
         <v>#REF!</v>
@@ -2830,11 +2827,11 @@
       <c r="I22" s="60"/>
       <c r="J22" s="103"/>
       <c r="K22" s="122"/>
-      <c r="L22" s="191" t="s">
+      <c r="L22" s="166" t="s">
         <v>54</v>
       </c>
-      <c r="M22" s="191"/>
-      <c r="N22" s="192"/>
+      <c r="M22" s="166"/>
+      <c r="N22" s="167"/>
       <c r="O22" s="58">
         <v>0</v>
       </c>
@@ -2849,9 +2846,9 @@
     <row r="23" spans="1:23" ht="45.75" customHeight="1">
       <c r="A23" s="65"/>
       <c r="B23" s="65"/>
-      <c r="C23" s="193"/>
-      <c r="D23" s="194"/>
-      <c r="E23" s="194"/>
+      <c r="C23" s="168"/>
+      <c r="D23" s="169"/>
+      <c r="E23" s="169"/>
       <c r="F23" s="130"/>
       <c r="G23" s="59" t="s">
         <v>22</v>
@@ -2878,9 +2875,9 @@
     <row r="24" spans="1:23" ht="45.75" customHeight="1">
       <c r="A24" s="65"/>
       <c r="B24" s="65"/>
-      <c r="C24" s="193"/>
-      <c r="D24" s="194"/>
-      <c r="E24" s="194"/>
+      <c r="C24" s="168"/>
+      <c r="D24" s="169"/>
+      <c r="E24" s="169"/>
       <c r="F24" s="58">
         <f>S14+S16</f>
         <v>0</v>
@@ -2910,9 +2907,9 @@
     <row r="25" spans="1:23" ht="45.75" customHeight="1">
       <c r="A25" s="65"/>
       <c r="B25" s="65"/>
-      <c r="C25" s="193"/>
-      <c r="D25" s="194"/>
-      <c r="E25" s="194"/>
+      <c r="C25" s="168"/>
+      <c r="D25" s="169"/>
+      <c r="E25" s="169"/>
       <c r="F25" s="58">
         <f>S15+S17</f>
         <v>0</v>
@@ -2942,9 +2939,9 @@
     <row r="26" spans="1:23" ht="45.75" customHeight="1">
       <c r="A26" s="65"/>
       <c r="B26" s="65"/>
-      <c r="C26" s="193"/>
-      <c r="D26" s="194"/>
-      <c r="E26" s="194"/>
+      <c r="C26" s="168"/>
+      <c r="D26" s="169"/>
+      <c r="E26" s="169"/>
       <c r="F26" s="58">
         <f>S18</f>
         <v>200000</v>
@@ -2997,39 +2994,39 @@
       <c r="W27" s="64"/>
     </row>
     <row r="28" spans="1:23" ht="51" customHeight="1">
-      <c r="A28" s="197" t="s">
+      <c r="A28" s="147" t="s">
         <v>41</v>
       </c>
-      <c r="B28" s="197"/>
-      <c r="C28" s="197"/>
-      <c r="D28" s="197" t="s">
+      <c r="B28" s="147"/>
+      <c r="C28" s="147"/>
+      <c r="D28" s="147" t="s">
         <v>6</v>
       </c>
-      <c r="E28" s="197"/>
-      <c r="F28" s="197"/>
-      <c r="G28" s="198" t="s">
+      <c r="E28" s="147"/>
+      <c r="F28" s="147"/>
+      <c r="G28" s="148" t="s">
         <v>7</v>
       </c>
-      <c r="H28" s="198"/>
+      <c r="H28" s="148"/>
       <c r="I28" s="66"/>
-      <c r="J28" s="197" t="s">
+      <c r="J28" s="147" t="s">
         <v>8</v>
       </c>
-      <c r="K28" s="197"/>
-      <c r="L28" s="197"/>
-      <c r="M28" s="197"/>
-      <c r="N28" s="197"/>
+      <c r="K28" s="147"/>
+      <c r="L28" s="147"/>
+      <c r="M28" s="147"/>
+      <c r="N28" s="147"/>
       <c r="O28" s="60"/>
       <c r="P28" s="70"/>
       <c r="Q28" s="82"/>
       <c r="R28" s="82"/>
       <c r="S28" s="82"/>
-      <c r="T28" s="199" t="s">
+      <c r="T28" s="149" t="s">
         <v>53</v>
       </c>
-      <c r="U28" s="199"/>
-      <c r="V28" s="199"/>
-      <c r="W28" s="199"/>
+      <c r="U28" s="149"/>
+      <c r="V28" s="149"/>
+      <c r="W28" s="149"/>
     </row>
     <row r="29" spans="1:23" ht="48.75" customHeight="1">
       <c r="A29" s="57"/>
@@ -3051,10 +3048,10 @@
       <c r="Q29" s="83"/>
       <c r="R29" s="83"/>
       <c r="S29" s="83"/>
-      <c r="T29" s="199"/>
-      <c r="U29" s="199"/>
-      <c r="V29" s="199"/>
-      <c r="W29" s="199"/>
+      <c r="T29" s="149"/>
+      <c r="U29" s="149"/>
+      <c r="V29" s="149"/>
+      <c r="W29" s="149"/>
     </row>
     <row r="30" spans="1:23" ht="58.2" customHeight="1">
       <c r="A30" s="57"/>
@@ -3076,10 +3073,10 @@
       <c r="Q30" s="83"/>
       <c r="R30" s="83"/>
       <c r="S30" s="83"/>
-      <c r="T30" s="199"/>
-      <c r="U30" s="199"/>
-      <c r="V30" s="199"/>
-      <c r="W30" s="199"/>
+      <c r="T30" s="149"/>
+      <c r="U30" s="149"/>
+      <c r="V30" s="149"/>
+      <c r="W30" s="149"/>
     </row>
     <row r="31" spans="1:23" ht="48.75" customHeight="1">
       <c r="A31" s="57"/>
@@ -3101,55 +3098,55 @@
       <c r="Q31" s="83"/>
       <c r="R31" s="83"/>
       <c r="S31" s="83"/>
-      <c r="T31" s="199"/>
-      <c r="U31" s="199"/>
-      <c r="V31" s="199"/>
-      <c r="W31" s="199"/>
+      <c r="T31" s="149"/>
+      <c r="U31" s="149"/>
+      <c r="V31" s="149"/>
+      <c r="W31" s="149"/>
     </row>
     <row r="32" spans="1:23" s="123" customFormat="1" ht="51.6" customHeight="1">
-      <c r="A32" s="152" t="e">
+      <c r="A32" s="183" t="e">
         <f>+C6</f>
         <v>#REF!</v>
       </c>
-      <c r="B32" s="152"/>
-      <c r="C32" s="152"/>
-      <c r="D32" s="153"/>
-      <c r="E32" s="153"/>
-      <c r="F32" s="153"/>
-      <c r="G32" s="154" t="s">
+      <c r="B32" s="183"/>
+      <c r="C32" s="183"/>
+      <c r="D32" s="184"/>
+      <c r="E32" s="184"/>
+      <c r="F32" s="184"/>
+      <c r="G32" s="185" t="s">
         <v>57</v>
       </c>
-      <c r="H32" s="154"/>
+      <c r="H32" s="185"/>
       <c r="I32" s="61"/>
-      <c r="J32" s="155"/>
-      <c r="K32" s="155"/>
-      <c r="L32" s="155"/>
-      <c r="M32" s="155"/>
-      <c r="N32" s="155"/>
+      <c r="J32" s="186"/>
+      <c r="K32" s="186"/>
+      <c r="L32" s="186"/>
+      <c r="M32" s="186"/>
+      <c r="N32" s="186"/>
       <c r="P32" s="64"/>
       <c r="Q32" s="88"/>
       <c r="R32" s="88"/>
       <c r="S32" s="88"/>
-      <c r="T32" s="199"/>
-      <c r="U32" s="199"/>
-      <c r="V32" s="199"/>
-      <c r="W32" s="199"/>
+      <c r="T32" s="149"/>
+      <c r="U32" s="149"/>
+      <c r="V32" s="149"/>
+      <c r="W32" s="149"/>
     </row>
     <row r="33" spans="1:23" ht="67.2" customHeight="1">
-      <c r="A33" s="182"/>
-      <c r="B33" s="182"/>
-      <c r="C33" s="182"/>
-      <c r="D33" s="183"/>
-      <c r="E33" s="183"/>
-      <c r="F33" s="183"/>
-      <c r="G33" s="184"/>
-      <c r="H33" s="184"/>
+      <c r="A33" s="150"/>
+      <c r="B33" s="150"/>
+      <c r="C33" s="150"/>
+      <c r="D33" s="151"/>
+      <c r="E33" s="151"/>
+      <c r="F33" s="151"/>
+      <c r="G33" s="152"/>
+      <c r="H33" s="152"/>
       <c r="I33" s="26"/>
-      <c r="J33" s="183"/>
-      <c r="K33" s="183"/>
-      <c r="L33" s="183"/>
-      <c r="M33" s="183"/>
-      <c r="N33" s="183"/>
+      <c r="J33" s="151"/>
+      <c r="K33" s="151"/>
+      <c r="L33" s="151"/>
+      <c r="M33" s="151"/>
+      <c r="N33" s="151"/>
       <c r="O33" s="40"/>
       <c r="P33" s="26"/>
       <c r="Q33" s="18"/>
@@ -3409,37 +3406,6 @@
     </row>
   </sheetData>
   <mergeCells count="46">
-    <mergeCell ref="V18:W18"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="D28:F28"/>
-    <mergeCell ref="G28:H28"/>
-    <mergeCell ref="J28:N28"/>
-    <mergeCell ref="T28:W32"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="D33:F33"/>
-    <mergeCell ref="G33:H33"/>
-    <mergeCell ref="J33:N33"/>
-    <mergeCell ref="Q17:R17"/>
-    <mergeCell ref="J16:L17"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="Q16:R16"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="L22:N22"/>
-    <mergeCell ref="C22:C26"/>
-    <mergeCell ref="D22:E26"/>
-    <mergeCell ref="Q18:R18"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="G1:W1"/>
-    <mergeCell ref="G2:W2"/>
-    <mergeCell ref="G3:W3"/>
-    <mergeCell ref="A4:W4"/>
-    <mergeCell ref="K5:N5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="F5:H5"/>
     <mergeCell ref="Q14:R14"/>
     <mergeCell ref="M15:N15"/>
     <mergeCell ref="L13:M13"/>
@@ -3455,6 +3421,37 @@
     <mergeCell ref="J14:L15"/>
     <mergeCell ref="M14:N14"/>
     <mergeCell ref="M18:N18"/>
+    <mergeCell ref="G1:W1"/>
+    <mergeCell ref="G2:W2"/>
+    <mergeCell ref="G3:W3"/>
+    <mergeCell ref="A4:W4"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="D33:F33"/>
+    <mergeCell ref="G33:H33"/>
+    <mergeCell ref="J33:N33"/>
+    <mergeCell ref="Q17:R17"/>
+    <mergeCell ref="J16:L17"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="Q16:R16"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="L22:N22"/>
+    <mergeCell ref="C22:C26"/>
+    <mergeCell ref="D22:E26"/>
+    <mergeCell ref="Q18:R18"/>
+    <mergeCell ref="V18:W18"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="J28:N28"/>
+    <mergeCell ref="T28:W32"/>
   </mergeCells>
   <phoneticPr fontId="26" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>